<commit_message>
Working 4-platform dashboard with URL mapping - pre search-first refactor
</commit_message>
<xml_diff>
--- a/data/sku_mapping.xlsx
+++ b/data/sku_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vacha\Desktop\I'\price-dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067995DF-7B42-4DD4-A5C9-BE2955939EE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EC9B69-EB36-4A6F-8BDD-25131B80E9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -658,7 +658,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -670,7 +670,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1010,6 +1009,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="41.88671875" customWidth="1"/>
+    <col min="3" max="3" width="34.77734375" customWidth="1"/>
+    <col min="4" max="4" width="37" customWidth="1"/>
+    <col min="5" max="5" width="25.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1062,7 +1064,7 @@
       <c r="B4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="1"/>

</xml_diff>